<commit_message>
Reorganise datasets from ecology_map to download_center
- Move all ecology_map/datasets/ GeoJSON, DEM, and source files to download_center/data/
- Remove ecology_map/README.md and ecology_map/downloadcentre.xlsx
- Update download_center/downloadcentre.xlsx
- Add root README.md

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/download_center/downloadcentre.xlsx
+++ b/download_center/downloadcentre.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\download_center\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92089F8C-63E0-4826-93D3-A14895E937CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3309D9F5-9A1A-4C26-9940-591C321DC786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="150" yWindow="1950" windowWidth="28650" windowHeight="15780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -126,9 +126,6 @@
     <t>/data/json/wetlands.geojson</t>
   </si>
   <si>
-    <t>/data/json/DEM.geojson</t>
-  </si>
-  <si>
     <t>/data/json/gba_wards.geojson</t>
   </si>
   <si>
@@ -232,6 +229,9 @@
   </si>
   <si>
     <t>/data/geotiff/cantonment_cog.tif</t>
+  </si>
+  <si>
+    <t>/data/geotiff/DEM.tif</t>
   </si>
 </sst>
 </file>
@@ -616,12 +616,12 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -635,7 +635,7 @@
     </row>
     <row r="3" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -649,7 +649,7 @@
     </row>
     <row r="4" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -663,7 +663,7 @@
     </row>
     <row r="5" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
@@ -677,7 +677,7 @@
     </row>
     <row r="6" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -691,64 +691,64 @@
     </row>
     <row r="7" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B11" t="s">
         <v>14</v>
@@ -762,7 +762,7 @@
     </row>
     <row r="12" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
         <v>7</v>
@@ -776,7 +776,7 @@
     </row>
     <row r="13" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
@@ -790,7 +790,7 @@
     </row>
     <row r="14" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
         <v>15</v>
@@ -804,7 +804,7 @@
     </row>
     <row r="15" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
         <v>10</v>
@@ -813,12 +813,12 @@
         <v>13</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
         <v>17</v>
@@ -832,7 +832,7 @@
     </row>
     <row r="17" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
         <v>18</v>
@@ -846,77 +846,77 @@
     </row>
     <row r="18" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" t="s">
         <v>55</v>
       </c>
-      <c r="B18" t="s">
-        <v>56</v>
-      </c>
       <c r="C18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="D19" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" t="s">
         <v>60</v>
       </c>
-      <c r="C20" t="s">
-        <v>61</v>
-      </c>
       <c r="D20" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" t="s">
         <v>63</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
         <v>8</v>
@@ -925,35 +925,35 @@
         <v>12</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" t="s">
         <v>49</v>
-      </c>
-      <c r="B24" t="s">
-        <v>50</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>